<commit_message>
Dashboard, Pages deploy, tests and MIT license
Also sums the bridge effects before subtracting them, and pins the workbook
timestamps so a rebuild gives identical bytes.
</commit_message>
<xml_diff>
--- a/output/defense_backlog_model.xlsx
+++ b/output/defense_backlog_model.xlsx
@@ -18664,7 +18664,7 @@
         <v/>
       </c>
       <c r="L2" s="5">
-        <f>(D2-C2)-I2-J2-K2</f>
+        <f>(D2-C2)-(I2+J2+K2)</f>
         <v/>
       </c>
     </row>
@@ -18714,7 +18714,7 @@
         <v/>
       </c>
       <c r="L3" s="5">
-        <f>(D3-C3)-I3-J3-K3</f>
+        <f>(D3-C3)-(I3+J3+K3)</f>
         <v/>
       </c>
     </row>
@@ -18764,7 +18764,7 @@
         <v/>
       </c>
       <c r="L4" s="5">
-        <f>(D4-C4)-I4-J4-K4</f>
+        <f>(D4-C4)-(I4+J4+K4)</f>
         <v/>
       </c>
     </row>
@@ -18814,7 +18814,7 @@
         <v/>
       </c>
       <c r="L5" s="5">
-        <f>(D5-C5)-I5-J5-K5</f>
+        <f>(D5-C5)-(I5+J5+K5)</f>
         <v/>
       </c>
     </row>
@@ -18864,7 +18864,7 @@
         <v/>
       </c>
       <c r="L6" s="5">
-        <f>(D6-C6)-I6-J6-K6</f>
+        <f>(D6-C6)-(I6+J6+K6)</f>
         <v/>
       </c>
     </row>
@@ -18914,7 +18914,7 @@
         <v/>
       </c>
       <c r="L7" s="5">
-        <f>(D7-C7)-I7-J7-K7</f>
+        <f>(D7-C7)-(I7+J7+K7)</f>
         <v/>
       </c>
     </row>
@@ -18964,7 +18964,7 @@
         <v/>
       </c>
       <c r="L8" s="5">
-        <f>(D8-C8)-I8-J8-K8</f>
+        <f>(D8-C8)-(I8+J8+K8)</f>
         <v/>
       </c>
     </row>
@@ -19014,7 +19014,7 @@
         <v/>
       </c>
       <c r="L9" s="5">
-        <f>(D9-C9)-I9-J9-K9</f>
+        <f>(D9-C9)-(I9+J9+K9)</f>
         <v/>
       </c>
     </row>
@@ -19064,7 +19064,7 @@
         <v/>
       </c>
       <c r="L10" s="5">
-        <f>(D10-C10)-I10-J10-K10</f>
+        <f>(D10-C10)-(I10+J10+K10)</f>
         <v/>
       </c>
     </row>
@@ -19114,7 +19114,7 @@
         <v/>
       </c>
       <c r="L11" s="5">
-        <f>(D11-C11)-I11-J11-K11</f>
+        <f>(D11-C11)-(I11+J11+K11)</f>
         <v/>
       </c>
     </row>
@@ -19164,7 +19164,7 @@
         <v/>
       </c>
       <c r="L12" s="5">
-        <f>(D12-C12)-I12-J12-K12</f>
+        <f>(D12-C12)-(I12+J12+K12)</f>
         <v/>
       </c>
     </row>
@@ -19214,7 +19214,7 @@
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>(D13-C13)-I13-J13-K13</f>
+        <f>(D13-C13)-(I13+J13+K13)</f>
         <v/>
       </c>
     </row>
@@ -19264,7 +19264,7 @@
         <v/>
       </c>
       <c r="L14" s="5">
-        <f>(D14-C14)-I14-J14-K14</f>
+        <f>(D14-C14)-(I14+J14+K14)</f>
         <v/>
       </c>
     </row>
@@ -19314,7 +19314,7 @@
         <v/>
       </c>
       <c r="L15" s="5">
-        <f>(D15-C15)-I15-J15-K15</f>
+        <f>(D15-C15)-(I15+J15+K15)</f>
         <v/>
       </c>
     </row>
@@ -19364,7 +19364,7 @@
         <v/>
       </c>
       <c r="L16" s="5">
-        <f>(D16-C16)-I16-J16-K16</f>
+        <f>(D16-C16)-(I16+J16+K16)</f>
         <v/>
       </c>
     </row>
@@ -19414,7 +19414,7 @@
         <v/>
       </c>
       <c r="L17" s="5">
-        <f>(D17-C17)-I17-J17-K17</f>
+        <f>(D17-C17)-(I17+J17+K17)</f>
         <v/>
       </c>
     </row>
@@ -19464,7 +19464,7 @@
         <v/>
       </c>
       <c r="L18" s="5">
-        <f>(D18-C18)-I18-J18-K18</f>
+        <f>(D18-C18)-(I18+J18+K18)</f>
         <v/>
       </c>
     </row>
@@ -19514,7 +19514,7 @@
         <v/>
       </c>
       <c r="L19" s="5">
-        <f>(D19-C19)-I19-J19-K19</f>
+        <f>(D19-C19)-(I19+J19+K19)</f>
         <v/>
       </c>
     </row>
@@ -19564,7 +19564,7 @@
         <v/>
       </c>
       <c r="L20" s="5">
-        <f>(D20-C20)-I20-J20-K20</f>
+        <f>(D20-C20)-(I20+J20+K20)</f>
         <v/>
       </c>
     </row>
@@ -19614,7 +19614,7 @@
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>(D21-C21)-I21-J21-K21</f>
+        <f>(D21-C21)-(I21+J21+K21)</f>
         <v/>
       </c>
     </row>
@@ -19664,7 +19664,7 @@
         <v/>
       </c>
       <c r="L22" s="5">
-        <f>(D22-C22)-I22-J22-K22</f>
+        <f>(D22-C22)-(I22+J22+K22)</f>
         <v/>
       </c>
     </row>
@@ -19714,7 +19714,7 @@
         <v/>
       </c>
       <c r="L23" s="5">
-        <f>(D23-C23)-I23-J23-K23</f>
+        <f>(D23-C23)-(I23+J23+K23)</f>
         <v/>
       </c>
     </row>
@@ -19764,7 +19764,7 @@
         <v/>
       </c>
       <c r="L24" s="5">
-        <f>(D24-C24)-I24-J24-K24</f>
+        <f>(D24-C24)-(I24+J24+K24)</f>
         <v/>
       </c>
     </row>
@@ -19814,7 +19814,7 @@
         <v/>
       </c>
       <c r="L25" s="5">
-        <f>(D25-C25)-I25-J25-K25</f>
+        <f>(D25-C25)-(I25+J25+K25)</f>
         <v/>
       </c>
     </row>
@@ -19864,7 +19864,7 @@
         <v/>
       </c>
       <c r="L26" s="5">
-        <f>(D26-C26)-I26-J26-K26</f>
+        <f>(D26-C26)-(I26+J26+K26)</f>
         <v/>
       </c>
     </row>
@@ -19914,7 +19914,7 @@
         <v/>
       </c>
       <c r="L27" s="5">
-        <f>(D27-C27)-I27-J27-K27</f>
+        <f>(D27-C27)-(I27+J27+K27)</f>
         <v/>
       </c>
     </row>

</xml_diff>